<commit_message>
voucher approval , sync pr to vouchers , purchase to export
</commit_message>
<xml_diff>
--- a/public/uploads/vouchers/Double_Voucher.xlsx
+++ b/public/uploads/vouchers/Double_Voucher.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Financial_System\financial-app\public\uploads\vouchers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEDBAE41-483A-49EB-80CD-5BDED4BB05A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D80601CF-4EB0-4FF3-AD3E-F3D9BD7EE286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -554,62 +554,34 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -620,25 +592,53 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1241,12 +1241,12 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
-      <c r="N4" s="33" t="s">
+      <c r="N4" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="O4" s="34"/>
-      <c r="P4" s="34"/>
-      <c r="Q4" s="35"/>
+      <c r="O4" s="47"/>
+      <c r="P4" s="47"/>
+      <c r="Q4" s="48"/>
       <c r="R4" s="8"/>
       <c r="S4" s="9" t="s">
         <v>3</v>
@@ -1276,12 +1276,12 @@
       <c r="K5" s="12"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
-      <c r="N5" s="36" t="s">
+      <c r="N5" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="O5" s="37"/>
-      <c r="P5" s="37"/>
-      <c r="Q5" s="38"/>
+      <c r="O5" s="34"/>
+      <c r="P5" s="34"/>
+      <c r="Q5" s="35"/>
       <c r="R5" s="13"/>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
@@ -1321,10 +1321,10 @@
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
-      <c r="N6" s="39"/>
-      <c r="O6" s="40"/>
-      <c r="P6" s="40"/>
-      <c r="Q6" s="41"/>
+      <c r="N6" s="65"/>
+      <c r="O6" s="42"/>
+      <c r="P6" s="42"/>
+      <c r="Q6" s="43"/>
       <c r="R6" s="13"/>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
@@ -1373,12 +1373,12 @@
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="43"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="43"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="37"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="37"/>
       <c r="K8" s="2"/>
       <c r="L8" s="18" t="s">
         <v>13</v>
@@ -1400,37 +1400,37 @@
       <c r="AA8" s="2"/>
     </row>
     <row r="9" spans="1:27" ht="18" customHeight="1">
-      <c r="A9" s="44" t="s">
+      <c r="A9" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="45" t="s">
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="38"/>
-      <c r="K9" s="57" t="s">
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="35"/>
+      <c r="K9" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="L9" s="59" t="s">
+      <c r="L9" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="M9" s="61" t="s">
+      <c r="M9" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="N9" s="37"/>
-      <c r="O9" s="37"/>
-      <c r="P9" s="37"/>
-      <c r="Q9" s="37"/>
-      <c r="R9" s="37"/>
-      <c r="S9" s="37"/>
-      <c r="T9" s="37"/>
-      <c r="U9" s="38"/>
+      <c r="N9" s="34"/>
+      <c r="O9" s="34"/>
+      <c r="P9" s="34"/>
+      <c r="Q9" s="34"/>
+      <c r="R9" s="34"/>
+      <c r="S9" s="34"/>
+      <c r="T9" s="34"/>
+      <c r="U9" s="35"/>
       <c r="V9" s="2"/>
       <c r="W9" s="2"/>
       <c r="X9" s="2"/>
@@ -1439,31 +1439,31 @@
       <c r="AA9" s="2"/>
     </row>
     <row r="10" spans="1:27" ht="18" customHeight="1">
-      <c r="A10" s="46" t="s">
+      <c r="A10" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="48" t="s">
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="43"/>
-      <c r="I10" s="43"/>
-      <c r="J10" s="47"/>
-      <c r="K10" s="58"/>
-      <c r="L10" s="58"/>
-      <c r="M10" s="62"/>
-      <c r="N10" s="43"/>
-      <c r="O10" s="43"/>
-      <c r="P10" s="43"/>
-      <c r="Q10" s="43"/>
-      <c r="R10" s="43"/>
-      <c r="S10" s="43"/>
-      <c r="T10" s="43"/>
-      <c r="U10" s="47"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="37"/>
+      <c r="J10" s="38"/>
+      <c r="K10" s="50"/>
+      <c r="L10" s="50"/>
+      <c r="M10" s="36"/>
+      <c r="N10" s="37"/>
+      <c r="O10" s="37"/>
+      <c r="P10" s="37"/>
+      <c r="Q10" s="37"/>
+      <c r="R10" s="37"/>
+      <c r="S10" s="37"/>
+      <c r="T10" s="37"/>
+      <c r="U10" s="38"/>
       <c r="V10" s="2"/>
       <c r="W10" s="2"/>
       <c r="X10" s="2"/>
@@ -1472,33 +1472,33 @@
       <c r="AA10" s="2"/>
     </row>
     <row r="11" spans="1:27" ht="12.75" customHeight="1">
-      <c r="A11" s="49" t="s">
+      <c r="A11" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="34"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="34"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="35"/>
-      <c r="K11" s="63" t="s">
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="47"/>
+      <c r="J11" s="48"/>
+      <c r="K11" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="L11" s="38"/>
-      <c r="M11" s="50" t="s">
+      <c r="L11" s="35"/>
+      <c r="M11" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="N11" s="34"/>
-      <c r="O11" s="34"/>
-      <c r="P11" s="34"/>
-      <c r="Q11" s="34"/>
-      <c r="R11" s="34"/>
-      <c r="S11" s="34"/>
-      <c r="T11" s="34"/>
-      <c r="U11" s="35"/>
+      <c r="N11" s="47"/>
+      <c r="O11" s="47"/>
+      <c r="P11" s="47"/>
+      <c r="Q11" s="47"/>
+      <c r="R11" s="47"/>
+      <c r="S11" s="47"/>
+      <c r="T11" s="47"/>
+      <c r="U11" s="48"/>
       <c r="V11" s="2"/>
       <c r="W11" s="2"/>
       <c r="X11" s="2"/>
@@ -1537,8 +1537,8 @@
       <c r="J12" s="19">
         <v>13</v>
       </c>
-      <c r="K12" s="62"/>
-      <c r="L12" s="47"/>
+      <c r="K12" s="36"/>
+      <c r="L12" s="38"/>
       <c r="M12" s="19">
         <v>16</v>
       </c>
@@ -1574,35 +1574,35 @@
       <c r="AA12" s="2"/>
     </row>
     <row r="13" spans="1:27" ht="24" customHeight="1">
-      <c r="A13" s="64" t="s">
+      <c r="A13" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="38"/>
-      <c r="K13" s="64" t="s">
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="34"/>
+      <c r="J13" s="35"/>
+      <c r="K13" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="L13" s="38"/>
-      <c r="M13" s="36" t="s">
+      <c r="L13" s="35"/>
+      <c r="M13" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="N13" s="38"/>
-      <c r="O13" s="66">
+      <c r="N13" s="35"/>
+      <c r="O13" s="68">
         <v>13195.09</v>
       </c>
-      <c r="P13" s="37"/>
-      <c r="Q13" s="37"/>
-      <c r="R13" s="37"/>
-      <c r="S13" s="37"/>
-      <c r="T13" s="37"/>
-      <c r="U13" s="38"/>
+      <c r="P13" s="34"/>
+      <c r="Q13" s="34"/>
+      <c r="R13" s="34"/>
+      <c r="S13" s="34"/>
+      <c r="T13" s="34"/>
+      <c r="U13" s="35"/>
       <c r="V13" s="15"/>
       <c r="W13" s="15"/>
       <c r="X13" s="15"/>
@@ -1611,70 +1611,64 @@
       <c r="AA13" s="15"/>
     </row>
     <row r="14" spans="1:27" ht="24" customHeight="1">
-      <c r="A14" s="65"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="40"/>
-      <c r="H14" s="40"/>
-      <c r="I14" s="40"/>
-      <c r="J14" s="41"/>
-      <c r="K14" s="62"/>
-      <c r="L14" s="47"/>
-      <c r="M14" s="62"/>
-      <c r="N14" s="47"/>
-      <c r="O14" s="62"/>
-      <c r="P14" s="43"/>
-      <c r="Q14" s="43"/>
-      <c r="R14" s="43"/>
-      <c r="S14" s="43"/>
-      <c r="T14" s="43"/>
-      <c r="U14" s="47"/>
+      <c r="A14" s="41"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="42"/>
+      <c r="J14" s="43"/>
+      <c r="K14" s="36"/>
+      <c r="L14" s="38"/>
+      <c r="M14" s="36"/>
+      <c r="N14" s="38"/>
+      <c r="O14" s="36"/>
+      <c r="P14" s="37"/>
+      <c r="Q14" s="37"/>
+      <c r="R14" s="37"/>
+      <c r="S14" s="37"/>
+      <c r="T14" s="37"/>
+      <c r="U14" s="38"/>
       <c r="V14" s="15"/>
-      <c r="W14" s="20">
-        <f>1374.37/0.12</f>
-        <v>11453.083333333299</v>
-      </c>
+      <c r="W14" s="15"/>
       <c r="X14" s="15"/>
       <c r="Y14" s="15"/>
       <c r="Z14" s="15"/>
       <c r="AA14" s="15"/>
     </row>
     <row r="15" spans="1:27" ht="24" customHeight="1">
-      <c r="A15" s="62"/>
-      <c r="B15" s="43"/>
-      <c r="C15" s="43"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="43"/>
-      <c r="I15" s="43"/>
-      <c r="J15" s="47"/>
-      <c r="K15" s="51" t="s">
+      <c r="A15" s="36"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="37"/>
+      <c r="J15" s="38"/>
+      <c r="K15" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="L15" s="35"/>
-      <c r="M15" s="52" t="s">
+      <c r="L15" s="48"/>
+      <c r="M15" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="N15" s="35"/>
-      <c r="O15" s="53">
+      <c r="N15" s="48"/>
+      <c r="O15" s="66">
         <v>9125.89</v>
       </c>
-      <c r="P15" s="34"/>
-      <c r="Q15" s="34"/>
-      <c r="R15" s="34"/>
-      <c r="S15" s="34"/>
-      <c r="T15" s="34"/>
-      <c r="U15" s="35"/>
+      <c r="P15" s="47"/>
+      <c r="Q15" s="47"/>
+      <c r="R15" s="47"/>
+      <c r="S15" s="47"/>
+      <c r="T15" s="47"/>
+      <c r="U15" s="48"/>
       <c r="V15" s="15"/>
-      <c r="W15" s="20">
-        <f>W14*1.12</f>
-        <v>12827.4533333333</v>
-      </c>
+      <c r="W15" s="15"/>
       <c r="X15" s="15"/>
       <c r="Y15" s="15"/>
       <c r="Z15" s="15"/>
@@ -1691,23 +1685,20 @@
       <c r="H16" s="21"/>
       <c r="I16" s="21"/>
       <c r="J16" s="21"/>
-      <c r="K16" s="54"/>
-      <c r="L16" s="35"/>
+      <c r="K16" s="53"/>
+      <c r="L16" s="48"/>
       <c r="M16" s="22"/>
       <c r="N16" s="23"/>
-      <c r="O16" s="53"/>
-      <c r="P16" s="34"/>
-      <c r="Q16" s="34"/>
-      <c r="R16" s="34"/>
-      <c r="S16" s="34"/>
-      <c r="T16" s="34"/>
-      <c r="U16" s="35"/>
+      <c r="O16" s="66"/>
+      <c r="P16" s="47"/>
+      <c r="Q16" s="47"/>
+      <c r="R16" s="47"/>
+      <c r="S16" s="47"/>
+      <c r="T16" s="47"/>
+      <c r="U16" s="48"/>
       <c r="V16" s="15"/>
       <c r="W16" s="15"/>
-      <c r="X16" s="15">
-        <f>12827.5-1374.37</f>
-        <v>11453.13</v>
-      </c>
+      <c r="X16" s="15"/>
       <c r="Y16" s="15"/>
       <c r="Z16" s="15"/>
       <c r="AA16" s="15"/>
@@ -1723,24 +1714,21 @@
       <c r="H17" s="21"/>
       <c r="I17" s="21"/>
       <c r="J17" s="21"/>
-      <c r="K17" s="54"/>
-      <c r="L17" s="35"/>
+      <c r="K17" s="53"/>
+      <c r="L17" s="48"/>
       <c r="M17" s="24"/>
       <c r="N17" s="25"/>
-      <c r="O17" s="55"/>
-      <c r="P17" s="34"/>
-      <c r="Q17" s="34"/>
-      <c r="R17" s="34"/>
-      <c r="S17" s="34"/>
-      <c r="T17" s="34"/>
-      <c r="U17" s="35"/>
+      <c r="O17" s="54"/>
+      <c r="P17" s="47"/>
+      <c r="Q17" s="47"/>
+      <c r="R17" s="47"/>
+      <c r="S17" s="47"/>
+      <c r="T17" s="47"/>
+      <c r="U17" s="48"/>
       <c r="V17" s="15"/>
       <c r="W17" s="15"/>
       <c r="X17" s="15"/>
-      <c r="Y17" s="15">
-        <f>4308/1.12</f>
-        <v>3846.4285714285702</v>
-      </c>
+      <c r="Y17" s="15"/>
       <c r="Z17" s="15"/>
       <c r="AA17" s="15"/>
     </row>
@@ -1755,58 +1743,55 @@
       <c r="H18" s="21"/>
       <c r="I18" s="21"/>
       <c r="J18" s="21"/>
-      <c r="K18" s="54"/>
-      <c r="L18" s="35"/>
+      <c r="K18" s="53"/>
+      <c r="L18" s="48"/>
       <c r="M18" s="24"/>
       <c r="N18" s="25"/>
-      <c r="O18" s="55"/>
-      <c r="P18" s="34"/>
-      <c r="Q18" s="34"/>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="35"/>
+      <c r="O18" s="54"/>
+      <c r="P18" s="47"/>
+      <c r="Q18" s="47"/>
+      <c r="R18" s="47"/>
+      <c r="S18" s="47"/>
+      <c r="T18" s="47"/>
+      <c r="U18" s="48"/>
       <c r="V18" s="15"/>
       <c r="W18" s="15"/>
       <c r="X18" s="15"/>
-      <c r="Y18" s="15">
-        <f>Y17*0.12</f>
-        <v>461.57142857142799</v>
-      </c>
+      <c r="Y18" s="15"/>
       <c r="Z18" s="15"/>
       <c r="AA18" s="26"/>
     </row>
     <row r="19" spans="1:27" ht="12.75" customHeight="1">
-      <c r="A19" s="49" t="s">
+      <c r="A19" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="34"/>
-      <c r="I19" s="34"/>
-      <c r="J19" s="35"/>
+      <c r="B19" s="47"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="47"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="47"/>
+      <c r="J19" s="48"/>
       <c r="K19" s="27"/>
-      <c r="L19" s="60" t="s">
+      <c r="L19" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="M19" s="64" t="s">
+      <c r="M19" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="N19" s="38"/>
-      <c r="O19" s="67">
+      <c r="N19" s="35"/>
+      <c r="O19" s="55">
         <f>SUM(O13:U18)</f>
         <v>22320.98</v>
       </c>
-      <c r="P19" s="37"/>
-      <c r="Q19" s="37"/>
-      <c r="R19" s="37"/>
-      <c r="S19" s="37"/>
-      <c r="T19" s="37"/>
-      <c r="U19" s="38"/>
+      <c r="P19" s="34"/>
+      <c r="Q19" s="34"/>
+      <c r="R19" s="34"/>
+      <c r="S19" s="34"/>
+      <c r="T19" s="34"/>
+      <c r="U19" s="35"/>
       <c r="V19" s="2"/>
       <c r="W19" s="2"/>
       <c r="X19" s="2"/>
@@ -1815,29 +1800,29 @@
       <c r="AA19" s="2"/>
     </row>
     <row r="20" spans="1:27" ht="12.75" customHeight="1">
-      <c r="A20" s="49" t="s">
+      <c r="A20" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="34"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="34"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="35"/>
+      <c r="B20" s="47"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="47"/>
+      <c r="F20" s="47"/>
+      <c r="G20" s="47"/>
+      <c r="H20" s="47"/>
+      <c r="I20" s="47"/>
+      <c r="J20" s="48"/>
       <c r="K20" s="28"/>
-      <c r="L20" s="47"/>
-      <c r="M20" s="62"/>
-      <c r="N20" s="47"/>
-      <c r="O20" s="62"/>
-      <c r="P20" s="43"/>
-      <c r="Q20" s="43"/>
-      <c r="R20" s="43"/>
-      <c r="S20" s="43"/>
-      <c r="T20" s="43"/>
-      <c r="U20" s="47"/>
+      <c r="L20" s="38"/>
+      <c r="M20" s="36"/>
+      <c r="N20" s="38"/>
+      <c r="O20" s="36"/>
+      <c r="P20" s="37"/>
+      <c r="Q20" s="37"/>
+      <c r="R20" s="37"/>
+      <c r="S20" s="37"/>
+      <c r="T20" s="37"/>
+      <c r="U20" s="38"/>
       <c r="V20" s="2"/>
       <c r="W20" s="2"/>
       <c r="X20" s="2"/>
@@ -1954,10 +1939,7 @@
       <c r="S24" s="2"/>
       <c r="T24" s="2"/>
       <c r="U24" s="2"/>
-      <c r="V24" s="30">
-        <f>O19+O43</f>
-        <v>24999.497599999999</v>
-      </c>
+      <c r="V24" s="2"/>
       <c r="W24" s="2"/>
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
@@ -2069,12 +2051,12 @@
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
-      <c r="N28" s="33" t="s">
+      <c r="N28" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="O28" s="34"/>
-      <c r="P28" s="34"/>
-      <c r="Q28" s="35"/>
+      <c r="O28" s="47"/>
+      <c r="P28" s="47"/>
+      <c r="Q28" s="48"/>
       <c r="R28" s="8"/>
       <c r="S28" s="9" t="s">
         <v>3</v>
@@ -2104,12 +2086,12 @@
       <c r="K29" s="12"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
-      <c r="N29" s="36" t="s">
+      <c r="N29" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="O29" s="37"/>
-      <c r="P29" s="37"/>
-      <c r="Q29" s="38"/>
+      <c r="O29" s="34"/>
+      <c r="P29" s="34"/>
+      <c r="Q29" s="35"/>
       <c r="R29" s="13"/>
       <c r="S29" s="2"/>
       <c r="T29" s="2"/>
@@ -2149,10 +2131,10 @@
       </c>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
-      <c r="N30" s="39"/>
-      <c r="O30" s="40"/>
-      <c r="P30" s="40"/>
-      <c r="Q30" s="41"/>
+      <c r="N30" s="65"/>
+      <c r="O30" s="42"/>
+      <c r="P30" s="42"/>
+      <c r="Q30" s="43"/>
       <c r="R30" s="13"/>
       <c r="S30" s="2"/>
       <c r="T30" s="2"/>
@@ -2201,12 +2183,12 @@
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
-      <c r="E32" s="42"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="43"/>
-      <c r="H32" s="43"/>
-      <c r="I32" s="43"/>
-      <c r="J32" s="43"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="37"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
@@ -2226,37 +2208,37 @@
       <c r="AA32" s="2"/>
     </row>
     <row r="33" spans="1:27" ht="18" customHeight="1">
-      <c r="A33" s="44" t="s">
+      <c r="A33" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="45" t="s">
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="35"/>
+      <c r="E33" s="61" t="s">
         <v>37</v>
       </c>
-      <c r="F33" s="37"/>
-      <c r="G33" s="37"/>
-      <c r="H33" s="37"/>
-      <c r="I33" s="37"/>
-      <c r="J33" s="38"/>
-      <c r="K33" s="57" t="s">
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="34"/>
+      <c r="I33" s="34"/>
+      <c r="J33" s="35"/>
+      <c r="K33" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="L33" s="59" t="s">
+      <c r="L33" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="M33" s="61" t="s">
+      <c r="M33" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="N33" s="37"/>
-      <c r="O33" s="37"/>
-      <c r="P33" s="37"/>
-      <c r="Q33" s="37"/>
-      <c r="R33" s="37"/>
-      <c r="S33" s="37"/>
-      <c r="T33" s="37"/>
-      <c r="U33" s="38"/>
+      <c r="N33" s="34"/>
+      <c r="O33" s="34"/>
+      <c r="P33" s="34"/>
+      <c r="Q33" s="34"/>
+      <c r="R33" s="34"/>
+      <c r="S33" s="34"/>
+      <c r="T33" s="34"/>
+      <c r="U33" s="35"/>
       <c r="V33" s="2"/>
       <c r="W33" s="2"/>
       <c r="X33" s="2"/>
@@ -2265,31 +2247,31 @@
       <c r="AA33" s="2"/>
     </row>
     <row r="34" spans="1:27" ht="18" customHeight="1">
-      <c r="A34" s="46" t="s">
+      <c r="A34" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="B34" s="43"/>
-      <c r="C34" s="43"/>
-      <c r="D34" s="47"/>
-      <c r="E34" s="48" t="s">
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="63" t="s">
         <v>39</v>
       </c>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="43"/>
-      <c r="I34" s="43"/>
-      <c r="J34" s="47"/>
-      <c r="K34" s="58"/>
-      <c r="L34" s="58"/>
-      <c r="M34" s="62"/>
-      <c r="N34" s="43"/>
-      <c r="O34" s="43"/>
-      <c r="P34" s="43"/>
-      <c r="Q34" s="43"/>
-      <c r="R34" s="43"/>
-      <c r="S34" s="43"/>
-      <c r="T34" s="43"/>
-      <c r="U34" s="47"/>
+      <c r="F34" s="37"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="37"/>
+      <c r="I34" s="37"/>
+      <c r="J34" s="38"/>
+      <c r="K34" s="50"/>
+      <c r="L34" s="50"/>
+      <c r="M34" s="36"/>
+      <c r="N34" s="37"/>
+      <c r="O34" s="37"/>
+      <c r="P34" s="37"/>
+      <c r="Q34" s="37"/>
+      <c r="R34" s="37"/>
+      <c r="S34" s="37"/>
+      <c r="T34" s="37"/>
+      <c r="U34" s="38"/>
       <c r="V34" s="2"/>
       <c r="W34" s="2"/>
       <c r="X34" s="2"/>
@@ -2298,33 +2280,33 @@
       <c r="AA34" s="2"/>
     </row>
     <row r="35" spans="1:27" ht="12.75" customHeight="1">
-      <c r="A35" s="49" t="s">
+      <c r="A35" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="34"/>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="34"/>
-      <c r="H35" s="34"/>
-      <c r="I35" s="34"/>
-      <c r="J35" s="35"/>
-      <c r="K35" s="63" t="s">
+      <c r="B35" s="47"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="47"/>
+      <c r="E35" s="47"/>
+      <c r="F35" s="47"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="47"/>
+      <c r="I35" s="47"/>
+      <c r="J35" s="48"/>
+      <c r="K35" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="L35" s="38"/>
-      <c r="M35" s="50" t="s">
+      <c r="L35" s="35"/>
+      <c r="M35" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="N35" s="34"/>
-      <c r="O35" s="34"/>
-      <c r="P35" s="34"/>
-      <c r="Q35" s="34"/>
-      <c r="R35" s="34"/>
-      <c r="S35" s="34"/>
-      <c r="T35" s="34"/>
-      <c r="U35" s="35"/>
+      <c r="N35" s="47"/>
+      <c r="O35" s="47"/>
+      <c r="P35" s="47"/>
+      <c r="Q35" s="47"/>
+      <c r="R35" s="47"/>
+      <c r="S35" s="47"/>
+      <c r="T35" s="47"/>
+      <c r="U35" s="48"/>
       <c r="V35" s="2"/>
       <c r="W35" s="2"/>
       <c r="X35" s="2"/>
@@ -2363,8 +2345,8 @@
       <c r="J36" s="19">
         <v>13</v>
       </c>
-      <c r="K36" s="62"/>
-      <c r="L36" s="47"/>
+      <c r="K36" s="36"/>
+      <c r="L36" s="38"/>
       <c r="M36" s="19">
         <v>16</v>
       </c>
@@ -2400,36 +2382,36 @@
       <c r="AA36" s="2"/>
     </row>
     <row r="37" spans="1:27" ht="24" customHeight="1">
-      <c r="A37" s="64" t="s">
+      <c r="A37" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="B37" s="37"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="37"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="37"/>
-      <c r="H37" s="37"/>
-      <c r="I37" s="37"/>
-      <c r="J37" s="38"/>
-      <c r="K37" s="64" t="s">
+      <c r="B37" s="34"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="34"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="34"/>
+      <c r="G37" s="34"/>
+      <c r="H37" s="34"/>
+      <c r="I37" s="34"/>
+      <c r="J37" s="35"/>
+      <c r="K37" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="L37" s="38"/>
-      <c r="M37" s="36" t="s">
+      <c r="L37" s="35"/>
+      <c r="M37" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="N37" s="38"/>
-      <c r="O37" s="68">
+      <c r="N37" s="35"/>
+      <c r="O37" s="45">
         <f>O13*0.12</f>
         <v>1583.4108000000001</v>
       </c>
-      <c r="P37" s="37"/>
-      <c r="Q37" s="37"/>
-      <c r="R37" s="37"/>
-      <c r="S37" s="37"/>
-      <c r="T37" s="37"/>
-      <c r="U37" s="38"/>
+      <c r="P37" s="34"/>
+      <c r="Q37" s="34"/>
+      <c r="R37" s="34"/>
+      <c r="S37" s="34"/>
+      <c r="T37" s="34"/>
+      <c r="U37" s="35"/>
       <c r="V37" s="15"/>
       <c r="W37" s="15"/>
       <c r="X37" s="15"/>
@@ -2438,27 +2420,27 @@
       <c r="AA37" s="15"/>
     </row>
     <row r="38" spans="1:27" ht="24" customHeight="1">
-      <c r="A38" s="65"/>
-      <c r="B38" s="40"/>
-      <c r="C38" s="40"/>
-      <c r="D38" s="40"/>
-      <c r="E38" s="40"/>
-      <c r="F38" s="40"/>
-      <c r="G38" s="40"/>
-      <c r="H38" s="40"/>
-      <c r="I38" s="40"/>
-      <c r="J38" s="41"/>
-      <c r="K38" s="62"/>
-      <c r="L38" s="47"/>
-      <c r="M38" s="62"/>
-      <c r="N38" s="47"/>
-      <c r="O38" s="62"/>
-      <c r="P38" s="43"/>
-      <c r="Q38" s="43"/>
-      <c r="R38" s="43"/>
-      <c r="S38" s="43"/>
-      <c r="T38" s="43"/>
-      <c r="U38" s="47"/>
+      <c r="A38" s="41"/>
+      <c r="B38" s="42"/>
+      <c r="C38" s="42"/>
+      <c r="D38" s="42"/>
+      <c r="E38" s="42"/>
+      <c r="F38" s="42"/>
+      <c r="G38" s="42"/>
+      <c r="H38" s="42"/>
+      <c r="I38" s="42"/>
+      <c r="J38" s="43"/>
+      <c r="K38" s="36"/>
+      <c r="L38" s="38"/>
+      <c r="M38" s="36"/>
+      <c r="N38" s="38"/>
+      <c r="O38" s="36"/>
+      <c r="P38" s="37"/>
+      <c r="Q38" s="37"/>
+      <c r="R38" s="37"/>
+      <c r="S38" s="37"/>
+      <c r="T38" s="37"/>
+      <c r="U38" s="38"/>
       <c r="V38" s="15"/>
       <c r="W38" s="15"/>
       <c r="X38" s="15"/>
@@ -2467,34 +2449,34 @@
       <c r="AA38" s="15"/>
     </row>
     <row r="39" spans="1:27" ht="24" customHeight="1">
-      <c r="A39" s="62"/>
-      <c r="B39" s="43"/>
-      <c r="C39" s="43"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="43"/>
-      <c r="I39" s="43"/>
-      <c r="J39" s="47"/>
-      <c r="K39" s="51" t="s">
+      <c r="A39" s="36"/>
+      <c r="B39" s="37"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="37"/>
+      <c r="E39" s="37"/>
+      <c r="F39" s="37"/>
+      <c r="G39" s="37"/>
+      <c r="H39" s="37"/>
+      <c r="I39" s="37"/>
+      <c r="J39" s="38"/>
+      <c r="K39" s="57" t="s">
         <v>41</v>
       </c>
-      <c r="L39" s="35"/>
+      <c r="L39" s="48"/>
       <c r="M39" s="24" t="s">
         <v>26</v>
       </c>
       <c r="N39" s="25"/>
-      <c r="O39" s="56">
+      <c r="O39" s="58">
         <f>O15*0.12</f>
         <v>1095.1068</v>
       </c>
-      <c r="P39" s="34"/>
-      <c r="Q39" s="34"/>
-      <c r="R39" s="34"/>
-      <c r="S39" s="34"/>
-      <c r="T39" s="34"/>
-      <c r="U39" s="35"/>
+      <c r="P39" s="47"/>
+      <c r="Q39" s="47"/>
+      <c r="R39" s="47"/>
+      <c r="S39" s="47"/>
+      <c r="T39" s="47"/>
+      <c r="U39" s="48"/>
       <c r="V39" s="15"/>
       <c r="W39" s="15"/>
       <c r="X39" s="15"/>
@@ -2513,17 +2495,17 @@
       <c r="H40" s="21"/>
       <c r="I40" s="21"/>
       <c r="J40" s="21"/>
-      <c r="K40" s="54"/>
-      <c r="L40" s="35"/>
+      <c r="K40" s="53"/>
+      <c r="L40" s="48"/>
       <c r="M40" s="24"/>
       <c r="N40" s="25"/>
-      <c r="O40" s="55"/>
-      <c r="P40" s="34"/>
-      <c r="Q40" s="34"/>
-      <c r="R40" s="34"/>
-      <c r="S40" s="34"/>
-      <c r="T40" s="34"/>
-      <c r="U40" s="35"/>
+      <c r="O40" s="54"/>
+      <c r="P40" s="47"/>
+      <c r="Q40" s="47"/>
+      <c r="R40" s="47"/>
+      <c r="S40" s="47"/>
+      <c r="T40" s="47"/>
+      <c r="U40" s="48"/>
       <c r="V40" s="15"/>
       <c r="W40" s="15"/>
       <c r="X40" s="15"/>
@@ -2542,17 +2524,17 @@
       <c r="H41" s="21"/>
       <c r="I41" s="21"/>
       <c r="J41" s="21"/>
-      <c r="K41" s="54"/>
-      <c r="L41" s="35"/>
+      <c r="K41" s="53"/>
+      <c r="L41" s="48"/>
       <c r="M41" s="24"/>
       <c r="N41" s="25"/>
-      <c r="O41" s="55"/>
-      <c r="P41" s="34"/>
-      <c r="Q41" s="34"/>
-      <c r="R41" s="34"/>
-      <c r="S41" s="34"/>
-      <c r="T41" s="34"/>
-      <c r="U41" s="35"/>
+      <c r="O41" s="54"/>
+      <c r="P41" s="47"/>
+      <c r="Q41" s="47"/>
+      <c r="R41" s="47"/>
+      <c r="S41" s="47"/>
+      <c r="T41" s="47"/>
+      <c r="U41" s="48"/>
       <c r="V41" s="15"/>
       <c r="W41" s="15"/>
       <c r="X41" s="15"/>
@@ -2571,17 +2553,17 @@
       <c r="H42" s="21"/>
       <c r="I42" s="21"/>
       <c r="J42" s="21"/>
-      <c r="K42" s="54"/>
-      <c r="L42" s="35"/>
+      <c r="K42" s="53"/>
+      <c r="L42" s="48"/>
       <c r="M42" s="24"/>
       <c r="N42" s="25"/>
-      <c r="O42" s="55"/>
-      <c r="P42" s="34"/>
-      <c r="Q42" s="34"/>
-      <c r="R42" s="34"/>
-      <c r="S42" s="34"/>
-      <c r="T42" s="34"/>
-      <c r="U42" s="35"/>
+      <c r="O42" s="54"/>
+      <c r="P42" s="47"/>
+      <c r="Q42" s="47"/>
+      <c r="R42" s="47"/>
+      <c r="S42" s="47"/>
+      <c r="T42" s="47"/>
+      <c r="U42" s="48"/>
       <c r="V42" s="15"/>
       <c r="W42" s="15"/>
       <c r="X42" s="15"/>
@@ -2590,37 +2572,37 @@
       <c r="AA42" s="15"/>
     </row>
     <row r="43" spans="1:27" ht="12.75" customHeight="1">
-      <c r="A43" s="49" t="s">
+      <c r="A43" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B43" s="34"/>
-      <c r="C43" s="34"/>
-      <c r="D43" s="34"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="34"/>
-      <c r="H43" s="34"/>
-      <c r="I43" s="34"/>
-      <c r="J43" s="35"/>
+      <c r="B43" s="47"/>
+      <c r="C43" s="47"/>
+      <c r="D43" s="47"/>
+      <c r="E43" s="47"/>
+      <c r="F43" s="47"/>
+      <c r="G43" s="47"/>
+      <c r="H43" s="47"/>
+      <c r="I43" s="47"/>
+      <c r="J43" s="48"/>
       <c r="K43" s="27"/>
-      <c r="L43" s="60" t="s">
+      <c r="L43" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="M43" s="64" t="str">
+      <c r="M43" s="40" t="str">
         <f>M37</f>
         <v>PHP</v>
       </c>
-      <c r="N43" s="38"/>
-      <c r="O43" s="67">
+      <c r="N43" s="35"/>
+      <c r="O43" s="55">
         <f>SUM(O37:U42)</f>
         <v>2678.5176000000001</v>
       </c>
-      <c r="P43" s="37"/>
-      <c r="Q43" s="37"/>
-      <c r="R43" s="37"/>
-      <c r="S43" s="37"/>
-      <c r="T43" s="37"/>
-      <c r="U43" s="38"/>
+      <c r="P43" s="34"/>
+      <c r="Q43" s="34"/>
+      <c r="R43" s="34"/>
+      <c r="S43" s="34"/>
+      <c r="T43" s="34"/>
+      <c r="U43" s="35"/>
       <c r="V43" s="2"/>
       <c r="W43" s="2"/>
       <c r="X43" s="2"/>
@@ -2629,29 +2611,29 @@
       <c r="AA43" s="2"/>
     </row>
     <row r="44" spans="1:27" ht="12.75" customHeight="1">
-      <c r="A44" s="49" t="s">
+      <c r="A44" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="B44" s="34"/>
-      <c r="C44" s="34"/>
-      <c r="D44" s="34"/>
-      <c r="E44" s="34"/>
-      <c r="F44" s="34"/>
-      <c r="G44" s="34"/>
-      <c r="H44" s="34"/>
-      <c r="I44" s="34"/>
-      <c r="J44" s="35"/>
+      <c r="B44" s="47"/>
+      <c r="C44" s="47"/>
+      <c r="D44" s="47"/>
+      <c r="E44" s="47"/>
+      <c r="F44" s="47"/>
+      <c r="G44" s="47"/>
+      <c r="H44" s="47"/>
+      <c r="I44" s="47"/>
+      <c r="J44" s="48"/>
       <c r="K44" s="28"/>
-      <c r="L44" s="47"/>
-      <c r="M44" s="62"/>
-      <c r="N44" s="47"/>
-      <c r="O44" s="62"/>
-      <c r="P44" s="43"/>
-      <c r="Q44" s="43"/>
-      <c r="R44" s="43"/>
-      <c r="S44" s="43"/>
-      <c r="T44" s="43"/>
-      <c r="U44" s="47"/>
+      <c r="L44" s="38"/>
+      <c r="M44" s="36"/>
+      <c r="N44" s="38"/>
+      <c r="O44" s="36"/>
+      <c r="P44" s="37"/>
+      <c r="Q44" s="37"/>
+      <c r="R44" s="37"/>
+      <c r="S44" s="37"/>
+      <c r="T44" s="37"/>
+      <c r="U44" s="38"/>
       <c r="V44" s="2"/>
       <c r="W44" s="2"/>
       <c r="X44" s="2"/>
@@ -30387,12 +30369,45 @@
     </row>
   </sheetData>
   <mergeCells count="63">
-    <mergeCell ref="M33:U34"/>
-    <mergeCell ref="K35:L36"/>
-    <mergeCell ref="A37:J39"/>
-    <mergeCell ref="K37:L38"/>
-    <mergeCell ref="M37:N38"/>
-    <mergeCell ref="O37:U38"/>
+    <mergeCell ref="N4:Q4"/>
+    <mergeCell ref="N5:Q5"/>
+    <mergeCell ref="N6:Q6"/>
+    <mergeCell ref="E8:J8"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="E9:J9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="E10:J10"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="M11:U11"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:U15"/>
+    <mergeCell ref="M9:U10"/>
+    <mergeCell ref="M13:N14"/>
+    <mergeCell ref="O13:U14"/>
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="O16:U16"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="O17:U17"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="O18:U18"/>
+    <mergeCell ref="N28:Q28"/>
+    <mergeCell ref="N29:Q29"/>
+    <mergeCell ref="N30:Q30"/>
+    <mergeCell ref="M19:N20"/>
+    <mergeCell ref="O19:U20"/>
+    <mergeCell ref="O40:U40"/>
+    <mergeCell ref="E32:J32"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="E33:J33"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="E34:J34"/>
+    <mergeCell ref="O41:U41"/>
+    <mergeCell ref="K42:L42"/>
+    <mergeCell ref="O42:U42"/>
+    <mergeCell ref="A43:J43"/>
+    <mergeCell ref="M43:N44"/>
+    <mergeCell ref="O43:U44"/>
     <mergeCell ref="A44:J44"/>
     <mergeCell ref="K9:K10"/>
     <mergeCell ref="K33:K34"/>
@@ -30404,52 +30419,19 @@
     <mergeCell ref="A13:J15"/>
     <mergeCell ref="K13:L14"/>
     <mergeCell ref="K41:L41"/>
-    <mergeCell ref="O41:U41"/>
-    <mergeCell ref="K42:L42"/>
-    <mergeCell ref="O42:U42"/>
-    <mergeCell ref="A43:J43"/>
-    <mergeCell ref="M43:N44"/>
-    <mergeCell ref="O43:U44"/>
     <mergeCell ref="A35:J35"/>
-    <mergeCell ref="M35:U35"/>
     <mergeCell ref="K39:L39"/>
-    <mergeCell ref="O39:U39"/>
     <mergeCell ref="K40:L40"/>
-    <mergeCell ref="O40:U40"/>
-    <mergeCell ref="E32:J32"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="E33:J33"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="E34:J34"/>
     <mergeCell ref="A19:J19"/>
     <mergeCell ref="A20:J20"/>
-    <mergeCell ref="N28:Q28"/>
-    <mergeCell ref="N29:Q29"/>
-    <mergeCell ref="N30:Q30"/>
-    <mergeCell ref="M19:N20"/>
-    <mergeCell ref="O19:U20"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="O16:U16"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="O17:U17"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="O18:U18"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="E10:J10"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="M11:U11"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:U15"/>
-    <mergeCell ref="M9:U10"/>
-    <mergeCell ref="M13:N14"/>
-    <mergeCell ref="O13:U14"/>
-    <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="N5:Q5"/>
-    <mergeCell ref="N6:Q6"/>
-    <mergeCell ref="E8:J8"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="E9:J9"/>
+    <mergeCell ref="M33:U34"/>
+    <mergeCell ref="K35:L36"/>
+    <mergeCell ref="A37:J39"/>
+    <mergeCell ref="K37:L38"/>
+    <mergeCell ref="M37:N38"/>
+    <mergeCell ref="O37:U38"/>
+    <mergeCell ref="M35:U35"/>
+    <mergeCell ref="O39:U39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>